<commit_message>
add objectType to truth matrix for Scoubi
</commit_message>
<xml_diff>
--- a/AdminSDHolderTruthMatrix.xlsx
+++ b/AdminSDHolderTruthMatrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Source\AdminSDHolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269DD0F3-4F1D-40F8-A054-AAF31AACA944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB12CDE2-11C5-46B5-B5F4-57E97AB6F9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40260" yWindow="1860" windowWidth="35020" windowHeight="18670" xr2:uid="{2AD1DF6E-F538-461F-9D50-BC6828A1C9AD}"/>
+    <workbookView xWindow="4820" yWindow="1110" windowWidth="35020" windowHeight="18670" xr2:uid="{2AD1DF6E-F538-461F-9D50-BC6828A1C9AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Version" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="116">
   <si>
     <t>Security Principal</t>
   </si>
@@ -367,6 +367,24 @@
   </si>
   <si>
     <t>BHE Tier0</t>
+  </si>
+  <si>
+    <t>Objectt Type</t>
+  </si>
+  <si>
+    <t>domainDNS</t>
+  </si>
+  <si>
+    <t>container</t>
+  </si>
+  <si>
+    <t>wellKnownSID</t>
+  </si>
+  <si>
+    <t>group</t>
+  </si>
+  <si>
+    <t>user</t>
   </si>
 </sst>
 </file>
@@ -441,7 +459,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -464,12 +482,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1"/>
@@ -516,6 +543,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -852,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79057642-481E-49F7-B76B-37B0532D9236}">
-  <dimension ref="A1:AJ68"/>
+  <dimension ref="A1:AK68"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.90625" bestFit="1" customWidth="1"/>
@@ -860,11 +893,12 @@
     <col min="3" max="3" width="13.7265625" style="5" customWidth="1"/>
     <col min="4" max="4" width="9" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.36328125" customWidth="1"/>
+    <col min="6" max="6" width="6" style="24" customWidth="1"/>
+    <col min="7" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="1" customFormat="1" ht="103.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" s="1" customFormat="1" ht="103.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -880,111 +914,114 @@
       <c r="E1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="J1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="M1" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="N1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="P1" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="Q1" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="R1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="S1" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="T1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="U1" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="V1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="W1" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="X1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="X1" s="10" t="s">
+      <c r="Y1" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="Y1" s="10" t="s">
+      <c r="Z1" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="Z1" s="10" t="s">
+      <c r="AA1" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="AA1" s="10" t="s">
+      <c r="AB1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AC1" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="AC1" s="19" t="s">
+      <c r="AD1" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="AD1" s="19" t="s">
+      <c r="AE1" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="AE1" s="19" t="s">
+      <c r="AF1" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="AF1" s="19" t="s">
+      <c r="AG1" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="AG1" s="19" t="s">
+      <c r="AH1" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="AH1" s="19" t="s">
+      <c r="AI1" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="AI1" s="19" t="s">
+      <c r="AJ1" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="AJ1" s="19" t="s">
+      <c r="AK1" s="19" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>56</v>
       </c>
-      <c r="S2" t="s">
-        <v>43</v>
+      <c r="F2" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T2" t="s">
         <v>43</v>
       </c>
-      <c r="V2" t="s">
+      <c r="U2" t="s">
         <v>43</v>
       </c>
       <c r="W2" t="s">
@@ -1002,8 +1039,11 @@
       <c r="AA2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1013,8 +1053,8 @@
       <c r="E3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>43</v>
+      <c r="F3" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>43</v>
@@ -1025,10 +1065,10 @@
       <c r="L3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M3" t="s">
-        <v>41</v>
-      </c>
-      <c r="O3" t="s">
+      <c r="M3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N3" t="s">
         <v>41</v>
       </c>
       <c r="P3" t="s">
@@ -1046,7 +1086,7 @@
       <c r="T3" t="s">
         <v>41</v>
       </c>
-      <c r="V3" t="s">
+      <c r="U3" t="s">
         <v>41</v>
       </c>
       <c r="W3" t="s">
@@ -1064,8 +1104,11 @@
       <c r="AA3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1075,8 +1118,8 @@
       <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>43</v>
+      <c r="F4" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>43</v>
@@ -1087,10 +1130,10 @@
       <c r="L4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M4" t="s">
-        <v>41</v>
-      </c>
-      <c r="O4" t="s">
+      <c r="M4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N4" t="s">
         <v>41</v>
       </c>
       <c r="P4" t="s">
@@ -1108,7 +1151,7 @@
       <c r="T4" t="s">
         <v>41</v>
       </c>
-      <c r="V4" t="s">
+      <c r="U4" t="s">
         <v>41</v>
       </c>
       <c r="W4" t="s">
@@ -1126,8 +1169,11 @@
       <c r="AA4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1137,8 +1183,8 @@
       <c r="E5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>43</v>
+      <c r="F5" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>43</v>
@@ -1149,10 +1195,10 @@
       <c r="L5" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O5" t="s">
+      <c r="M5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N5" t="s">
         <v>41</v>
       </c>
       <c r="P5" t="s">
@@ -1170,7 +1216,7 @@
       <c r="T5" t="s">
         <v>41</v>
       </c>
-      <c r="V5" t="s">
+      <c r="U5" t="s">
         <v>41</v>
       </c>
       <c r="W5" t="s">
@@ -1188,13 +1234,16 @@
       <c r="AA5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>57</v>
       </c>
-      <c r="Q6" t="s">
-        <v>43</v>
+      <c r="F6" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R6" t="s">
         <v>43</v>
@@ -1205,7 +1254,7 @@
       <c r="T6" t="s">
         <v>43</v>
       </c>
-      <c r="V6" t="s">
+      <c r="U6" t="s">
         <v>43</v>
       </c>
       <c r="W6" t="s">
@@ -1223,16 +1272,19 @@
       <c r="AA6" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>76</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="Q7" t="s">
-        <v>43</v>
+      <c r="F7" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R7" t="s">
         <v>43</v>
@@ -1243,7 +1295,7 @@
       <c r="T7" t="s">
         <v>43</v>
       </c>
-      <c r="V7" t="s">
+      <c r="U7" t="s">
         <v>43</v>
       </c>
       <c r="W7" t="s">
@@ -1261,16 +1313,19 @@
       <c r="AA7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>42</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="O8" t="s">
-        <v>43</v>
+      <c r="F8" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P8" t="s">
         <v>43</v>
@@ -1287,7 +1342,7 @@
       <c r="T8" t="s">
         <v>43</v>
       </c>
-      <c r="V8" t="s">
+      <c r="U8" t="s">
         <v>43</v>
       </c>
       <c r="W8" t="s">
@@ -1305,13 +1360,16 @@
       <c r="AA8" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>77</v>
       </c>
-      <c r="Q9" t="s">
-        <v>43</v>
+      <c r="F9" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R9" t="s">
         <v>43</v>
@@ -1322,7 +1380,7 @@
       <c r="T9" t="s">
         <v>43</v>
       </c>
-      <c r="V9" t="s">
+      <c r="U9" t="s">
         <v>43</v>
       </c>
       <c r="W9" t="s">
@@ -1340,18 +1398,21 @@
       <c r="AA9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>58</v>
       </c>
-      <c r="S10" t="s">
-        <v>43</v>
+      <c r="F10" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T10" t="s">
         <v>43</v>
       </c>
-      <c r="V10" t="s">
+      <c r="U10" t="s">
         <v>43</v>
       </c>
       <c r="W10" t="s">
@@ -1369,13 +1430,16 @@
       <c r="AA10" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>75</v>
       </c>
-      <c r="Q11" t="s">
-        <v>43</v>
+      <c r="F11" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R11" t="s">
         <v>43</v>
@@ -1386,7 +1450,7 @@
       <c r="T11" t="s">
         <v>43</v>
       </c>
-      <c r="V11" t="s">
+      <c r="U11" t="s">
         <v>43</v>
       </c>
       <c r="W11" t="s">
@@ -1404,13 +1468,16 @@
       <c r="AA11" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>44</v>
       </c>
-      <c r="O12" t="s">
-        <v>43</v>
+      <c r="F12" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P12" t="s">
         <v>43</v>
@@ -1427,7 +1494,7 @@
       <c r="T12" t="s">
         <v>43</v>
       </c>
-      <c r="V12" t="s">
+      <c r="U12" t="s">
         <v>43</v>
       </c>
       <c r="W12" t="s">
@@ -1445,13 +1512,16 @@
       <c r="AA12" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>45</v>
       </c>
-      <c r="O13" t="s">
-        <v>43</v>
+      <c r="F13" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P13" t="s">
         <v>43</v>
@@ -1468,7 +1538,7 @@
       <c r="T13" t="s">
         <v>43</v>
       </c>
-      <c r="V13" t="s">
+      <c r="U13" t="s">
         <v>43</v>
       </c>
       <c r="W13" t="s">
@@ -1486,24 +1556,30 @@
       <c r="AA13" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>59</v>
       </c>
-      <c r="Y14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="F14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="O15" t="s">
-        <v>43</v>
+      <c r="F15" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P15" t="s">
         <v>43</v>
@@ -1520,7 +1596,7 @@
       <c r="T15" t="s">
         <v>43</v>
       </c>
-      <c r="V15" t="s">
+      <c r="U15" t="s">
         <v>43</v>
       </c>
       <c r="W15" t="s">
@@ -1538,13 +1614,16 @@
       <c r="AA15" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+      <c r="AB15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>47</v>
       </c>
-      <c r="O16" t="s">
-        <v>43</v>
+      <c r="F16" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P16" t="s">
         <v>43</v>
@@ -1561,7 +1640,7 @@
       <c r="T16" t="s">
         <v>43</v>
       </c>
-      <c r="V16" t="s">
+      <c r="U16" t="s">
         <v>43</v>
       </c>
       <c r="W16" t="s">
@@ -1579,13 +1658,16 @@
       <c r="AA16" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="I17" t="s">
-        <v>43</v>
+      <c r="F17" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J17" t="s">
         <v>43</v>
@@ -1599,7 +1681,7 @@
       <c r="M17" t="s">
         <v>43</v>
       </c>
-      <c r="O17" t="s">
+      <c r="N17" t="s">
         <v>43</v>
       </c>
       <c r="P17" t="s">
@@ -1617,7 +1699,7 @@
       <c r="T17" t="s">
         <v>43</v>
       </c>
-      <c r="V17" t="s">
+      <c r="U17" t="s">
         <v>43</v>
       </c>
       <c r="W17" t="s">
@@ -1635,8 +1717,11 @@
       <c r="AA17" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -1646,8 +1731,8 @@
       <c r="E18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="3" t="s">
-        <v>43</v>
+      <c r="F18" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>43</v>
@@ -1658,10 +1743,10 @@
       <c r="L18" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M18" t="s">
-        <v>41</v>
-      </c>
-      <c r="O18" t="s">
+      <c r="M18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N18" t="s">
         <v>41</v>
       </c>
       <c r="P18" t="s">
@@ -1679,7 +1764,7 @@
       <c r="T18" t="s">
         <v>41</v>
       </c>
-      <c r="V18" t="s">
+      <c r="U18" t="s">
         <v>41</v>
       </c>
       <c r="W18" t="s">
@@ -1697,18 +1782,21 @@
       <c r="AA18" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>60</v>
       </c>
-      <c r="S19" t="s">
-        <v>43</v>
+      <c r="F19" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T19" t="s">
         <v>43</v>
       </c>
-      <c r="V19" t="s">
+      <c r="U19" t="s">
         <v>43</v>
       </c>
       <c r="W19" t="s">
@@ -1726,18 +1814,21 @@
       <c r="AA19" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>61</v>
       </c>
-      <c r="S20" t="s">
-        <v>43</v>
+      <c r="F20" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T20" t="s">
         <v>43</v>
       </c>
-      <c r="V20" t="s">
+      <c r="U20" t="s">
         <v>43</v>
       </c>
       <c r="W20" t="s">
@@ -1755,18 +1846,21 @@
       <c r="AA20" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>62</v>
       </c>
-      <c r="S21" t="s">
-        <v>43</v>
+      <c r="F21" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T21" t="s">
         <v>43</v>
       </c>
-      <c r="V21" t="s">
+      <c r="U21" t="s">
         <v>43</v>
       </c>
       <c r="W21" t="s">
@@ -1784,13 +1878,16 @@
       <c r="AA21" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="O22" t="s">
-        <v>43</v>
+      <c r="F22" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P22" t="s">
         <v>43</v>
@@ -1807,7 +1904,7 @@
       <c r="T22" t="s">
         <v>43</v>
       </c>
-      <c r="V22" t="s">
+      <c r="U22" t="s">
         <v>43</v>
       </c>
       <c r="W22" t="s">
@@ -1825,18 +1922,21 @@
       <c r="AA22" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>63</v>
       </c>
-      <c r="S23" t="s">
-        <v>43</v>
+      <c r="F23" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T23" t="s">
         <v>43</v>
       </c>
-      <c r="V23" t="s">
+      <c r="U23" t="s">
         <v>43</v>
       </c>
       <c r="W23" t="s">
@@ -1854,13 +1954,16 @@
       <c r="AA23" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
-      <c r="I24" t="s">
-        <v>43</v>
+      <c r="F24" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J24" t="s">
         <v>43</v>
@@ -1872,9 +1975,9 @@
         <v>43</v>
       </c>
       <c r="M24" t="s">
-        <v>41</v>
-      </c>
-      <c r="O24" t="s">
+        <v>43</v>
+      </c>
+      <c r="N24" t="s">
         <v>41</v>
       </c>
       <c r="P24" t="s">
@@ -1892,7 +1995,7 @@
       <c r="T24" t="s">
         <v>41</v>
       </c>
-      <c r="V24" t="s">
+      <c r="U24" t="s">
         <v>41</v>
       </c>
       <c r="W24" t="s">
@@ -1910,8 +2013,11 @@
       <c r="AA24" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB24" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1921,8 +2027,8 @@
       <c r="E25" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>43</v>
+      <c r="F25" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>43</v>
@@ -1933,10 +2039,10 @@
       <c r="L25" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M25" t="s">
-        <v>41</v>
-      </c>
-      <c r="O25" t="s">
+      <c r="M25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N25" t="s">
         <v>41</v>
       </c>
       <c r="P25" t="s">
@@ -1954,7 +2060,7 @@
       <c r="T25" t="s">
         <v>41</v>
       </c>
-      <c r="V25" t="s">
+      <c r="U25" t="s">
         <v>41</v>
       </c>
       <c r="W25" t="s">
@@ -1972,13 +2078,16 @@
       <c r="AA25" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>64</v>
       </c>
-      <c r="V26" t="s">
-        <v>43</v>
+      <c r="F26" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="W26" t="s">
         <v>43</v>
@@ -1995,13 +2104,16 @@
       <c r="AA26" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB26" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>49</v>
       </c>
-      <c r="O27" t="s">
-        <v>43</v>
+      <c r="F27" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P27" t="s">
         <v>43</v>
@@ -2018,7 +2130,7 @@
       <c r="T27" t="s">
         <v>43</v>
       </c>
-      <c r="V27" t="s">
+      <c r="U27" t="s">
         <v>43</v>
       </c>
       <c r="W27" t="s">
@@ -2036,13 +2148,16 @@
       <c r="AA27" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB27" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>50</v>
       </c>
-      <c r="O28" t="s">
-        <v>43</v>
+      <c r="F28" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P28" t="s">
         <v>43</v>
@@ -2059,7 +2174,7 @@
       <c r="T28" t="s">
         <v>43</v>
       </c>
-      <c r="V28" t="s">
+      <c r="U28" t="s">
         <v>43</v>
       </c>
       <c r="W28" t="s">
@@ -2077,8 +2192,11 @@
       <c r="AA28" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB28" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -2088,8 +2206,8 @@
       <c r="C29" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I29" t="s">
-        <v>41</v>
+      <c r="F29" s="24" t="s">
+        <v>115</v>
       </c>
       <c r="J29" t="s">
         <v>41</v>
@@ -2103,7 +2221,7 @@
       <c r="M29" t="s">
         <v>41</v>
       </c>
-      <c r="O29" t="s">
+      <c r="N29" t="s">
         <v>41</v>
       </c>
       <c r="P29" t="s">
@@ -2121,7 +2239,7 @@
       <c r="T29" t="s">
         <v>41</v>
       </c>
-      <c r="V29" t="s">
+      <c r="U29" t="s">
         <v>41</v>
       </c>
       <c r="W29" t="s">
@@ -2139,16 +2257,19 @@
       <c r="AA29" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB29" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>65</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="Q30" t="s">
-        <v>43</v>
+      <c r="F30" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R30" t="s">
         <v>43</v>
@@ -2159,7 +2280,7 @@
       <c r="T30" t="s">
         <v>43</v>
       </c>
-      <c r="V30" t="s">
+      <c r="U30" t="s">
         <v>43</v>
       </c>
       <c r="W30" t="s">
@@ -2177,16 +2298,19 @@
       <c r="AA30" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>3</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I31" s="3" t="s">
-        <v>43</v>
+      <c r="F31" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>43</v>
@@ -2197,14 +2321,14 @@
       <c r="L31" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M31" t="s">
-        <v>41</v>
-      </c>
-      <c r="N31" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="O31" s="3" t="s">
-        <v>43</v>
+      <c r="M31" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N31" t="s">
+        <v>41</v>
+      </c>
+      <c r="O31" s="6" t="s">
+        <v>41</v>
       </c>
       <c r="P31" s="3" t="s">
         <v>43</v>
@@ -2221,10 +2345,10 @@
       <c r="T31" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="U31" s="3"/>
-      <c r="V31" s="3" t="s">
-        <v>43</v>
-      </c>
+      <c r="U31" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="V31" s="3"/>
       <c r="W31" s="3" t="s">
         <v>43</v>
       </c>
@@ -2240,18 +2364,21 @@
       <c r="AA31" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB31" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>66</v>
       </c>
-      <c r="S32" t="s">
-        <v>43</v>
+      <c r="F32" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="T32" t="s">
         <v>43</v>
       </c>
-      <c r="V32" t="s">
+      <c r="U32" t="s">
         <v>43</v>
       </c>
       <c r="W32" t="s">
@@ -2269,16 +2396,19 @@
       <c r="AA32" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB32" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>67</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="Q33" t="s">
-        <v>43</v>
+      <c r="F33" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R33" t="s">
         <v>43</v>
@@ -2289,7 +2419,7 @@
       <c r="T33" t="s">
         <v>43</v>
       </c>
-      <c r="V33" t="s">
+      <c r="U33" t="s">
         <v>43</v>
       </c>
       <c r="W33" t="s">
@@ -2307,16 +2437,19 @@
       <c r="AA33" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB33" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>4</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I34" s="3" t="s">
-        <v>43</v>
+      <c r="F34" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>43</v>
@@ -2330,7 +2463,7 @@
       <c r="M34" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="O34" s="3" t="s">
+      <c r="N34" s="3" t="s">
         <v>43</v>
       </c>
       <c r="P34" s="3" t="s">
@@ -2348,10 +2481,10 @@
       <c r="T34" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="U34" s="3"/>
-      <c r="V34" s="3" t="s">
-        <v>43</v>
-      </c>
+      <c r="U34" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="V34" s="3"/>
       <c r="W34" s="3" t="s">
         <v>43</v>
       </c>
@@ -2367,13 +2500,16 @@
       <c r="AA34" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB34" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>9</v>
       </c>
-      <c r="I35" t="s">
-        <v>43</v>
+      <c r="F35" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J35" t="s">
         <v>43</v>
@@ -2387,7 +2523,7 @@
       <c r="M35" t="s">
         <v>43</v>
       </c>
-      <c r="O35" t="s">
+      <c r="N35" t="s">
         <v>43</v>
       </c>
       <c r="P35" t="s">
@@ -2405,7 +2541,7 @@
       <c r="T35" t="s">
         <v>43</v>
       </c>
-      <c r="V35" t="s">
+      <c r="U35" t="s">
         <v>43</v>
       </c>
       <c r="W35" t="s">
@@ -2423,8 +2559,11 @@
       <c r="AA35" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -2434,8 +2573,8 @@
       <c r="C36" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I36" t="s">
-        <v>41</v>
+      <c r="F36" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J36" t="s">
         <v>41</v>
@@ -2449,7 +2588,7 @@
       <c r="M36" t="s">
         <v>41</v>
       </c>
-      <c r="O36" t="s">
+      <c r="N36" t="s">
         <v>41</v>
       </c>
       <c r="P36" t="s">
@@ -2467,7 +2606,7 @@
       <c r="T36" t="s">
         <v>41</v>
       </c>
-      <c r="V36" t="s">
+      <c r="U36" t="s">
         <v>41</v>
       </c>
       <c r="W36" t="s">
@@ -2485,8 +2624,11 @@
       <c r="AA36" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB36" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -2499,8 +2641,8 @@
       <c r="D37" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="I37" s="3" t="s">
-        <v>43</v>
+      <c r="F37" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J37" s="3" t="s">
         <v>43</v>
@@ -2511,10 +2653,10 @@
       <c r="L37" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M37" t="s">
-        <v>41</v>
-      </c>
-      <c r="O37" t="s">
+      <c r="M37" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N37" t="s">
         <v>41</v>
       </c>
       <c r="P37" t="s">
@@ -2532,7 +2674,7 @@
       <c r="T37" t="s">
         <v>41</v>
       </c>
-      <c r="V37" t="s">
+      <c r="U37" t="s">
         <v>41</v>
       </c>
       <c r="W37" t="s">
@@ -2550,8 +2692,11 @@
       <c r="AA37" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB37" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="38" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>7</v>
       </c>
@@ -2561,8 +2706,8 @@
       <c r="C38" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I38" t="s">
-        <v>41</v>
+      <c r="F38" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J38" t="s">
         <v>41</v>
@@ -2576,7 +2721,7 @@
       <c r="M38" t="s">
         <v>41</v>
       </c>
-      <c r="O38" t="s">
+      <c r="N38" t="s">
         <v>41</v>
       </c>
       <c r="P38" t="s">
@@ -2594,7 +2739,7 @@
       <c r="T38" t="s">
         <v>41</v>
       </c>
-      <c r="V38" t="s">
+      <c r="U38" t="s">
         <v>41</v>
       </c>
       <c r="W38" t="s">
@@ -2612,8 +2757,11 @@
       <c r="AA38" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB38" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="39" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>68</v>
       </c>
@@ -2623,11 +2771,11 @@
       <c r="C39" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="V39" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="W39" t="s">
-        <v>41</v>
+      <c r="F39" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="W39" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="X39" t="s">
         <v>41</v>
@@ -2641,16 +2789,19 @@
       <c r="AA39" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB39" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="40" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>69</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="Q40" t="s">
-        <v>43</v>
+      <c r="F40" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R40" t="s">
         <v>43</v>
@@ -2661,7 +2812,7 @@
       <c r="T40" t="s">
         <v>43</v>
       </c>
-      <c r="V40" t="s">
+      <c r="U40" t="s">
         <v>43</v>
       </c>
       <c r="W40" t="s">
@@ -2679,32 +2830,41 @@
       <c r="AA40" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB40" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>70</v>
       </c>
-      <c r="Y41" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F41" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>71</v>
       </c>
-      <c r="Y42" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="43" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F42" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="I43" t="s">
-        <v>43</v>
+      <c r="F43" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J43" t="s">
         <v>43</v>
@@ -2718,7 +2878,7 @@
       <c r="M43" t="s">
         <v>43</v>
       </c>
-      <c r="O43" t="s">
+      <c r="N43" t="s">
         <v>43</v>
       </c>
       <c r="P43" t="s">
@@ -2736,7 +2896,7 @@
       <c r="T43" t="s">
         <v>43</v>
       </c>
-      <c r="V43" t="s">
+      <c r="U43" t="s">
         <v>43</v>
       </c>
       <c r="W43" t="s">
@@ -2754,19 +2914,25 @@
       <c r="AA43" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="44" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB43" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="44" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>51</v>
       </c>
-      <c r="O44" t="s">
-        <v>43</v>
+      <c r="F44" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P44" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="Q44" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>72</v>
       </c>
@@ -2776,10 +2942,10 @@
       <c r="C45" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="V45" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="W45" t="s">
+      <c r="F45" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="W45" s="6" t="s">
         <v>41</v>
       </c>
       <c r="X45" t="s">
@@ -2794,8 +2960,11 @@
       <c r="AA45" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="46" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB45" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>10</v>
       </c>
@@ -2803,8 +2972,8 @@
       <c r="C46" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I46" s="4" t="s">
-        <v>43</v>
+      <c r="F46" s="24" t="s">
+        <v>115</v>
       </c>
       <c r="J46" s="4" t="s">
         <v>43</v>
@@ -2815,10 +2984,10 @@
       <c r="L46" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="M46" t="s">
-        <v>41</v>
-      </c>
-      <c r="O46" t="s">
+      <c r="M46" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N46" t="s">
         <v>41</v>
       </c>
       <c r="P46" t="s">
@@ -2836,7 +3005,7 @@
       <c r="T46" t="s">
         <v>41</v>
       </c>
-      <c r="V46" t="s">
+      <c r="U46" t="s">
         <v>41</v>
       </c>
       <c r="W46" t="s">
@@ -2854,16 +3023,19 @@
       <c r="AA46" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="47" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB46" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>73</v>
       </c>
-      <c r="I47" s="2"/>
-      <c r="T47" t="s">
-        <v>43</v>
-      </c>
-      <c r="V47" t="s">
+      <c r="F47" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="J47" s="2"/>
+      <c r="U47" t="s">
         <v>43</v>
       </c>
       <c r="W47" t="s">
@@ -2881,13 +3053,16 @@
       <c r="AA47" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="48" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB47" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>11</v>
       </c>
-      <c r="I48" t="s">
-        <v>43</v>
+      <c r="F48" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J48" t="s">
         <v>43</v>
@@ -2901,7 +3076,7 @@
       <c r="M48" t="s">
         <v>43</v>
       </c>
-      <c r="O48" t="s">
+      <c r="N48" t="s">
         <v>43</v>
       </c>
       <c r="P48" t="s">
@@ -2919,7 +3094,7 @@
       <c r="T48" t="s">
         <v>43</v>
       </c>
-      <c r="V48" t="s">
+      <c r="U48" t="s">
         <v>43</v>
       </c>
       <c r="W48" t="s">
@@ -2937,8 +3112,11 @@
       <c r="AA48" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="49" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB48" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>74</v>
       </c>
@@ -2948,8 +3126,8 @@
       <c r="D49" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="Q49" t="s">
-        <v>41</v>
+      <c r="F49" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="R49" t="s">
         <v>41</v>
@@ -2960,7 +3138,7 @@
       <c r="T49" t="s">
         <v>41</v>
       </c>
-      <c r="V49" t="s">
+      <c r="U49" t="s">
         <v>41</v>
       </c>
       <c r="W49" t="s">
@@ -2978,8 +3156,11 @@
       <c r="AA49" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="50" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB49" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>12</v>
       </c>
@@ -2989,8 +3170,8 @@
       <c r="C50" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I50" t="s">
-        <v>41</v>
+      <c r="F50" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="J50" t="s">
         <v>41</v>
@@ -3004,7 +3185,7 @@
       <c r="M50" t="s">
         <v>41</v>
       </c>
-      <c r="O50" t="s">
+      <c r="N50" t="s">
         <v>41</v>
       </c>
       <c r="P50" t="s">
@@ -3022,7 +3203,7 @@
       <c r="T50" t="s">
         <v>41</v>
       </c>
-      <c r="V50" t="s">
+      <c r="U50" t="s">
         <v>41</v>
       </c>
       <c r="W50" t="s">
@@ -3040,43 +3221,58 @@
       <c r="AA50" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="51" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB50" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>79</v>
       </c>
-      <c r="T51" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="52" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F51" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="U51" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>52</v>
       </c>
-      <c r="O52" t="s">
-        <v>43</v>
+      <c r="F52" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="P52" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="53" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="Q52" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>85</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="54" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F53" s="24" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="54" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>86</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="55" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F54" s="24" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="55" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>106</v>
       </c>
@@ -3086,8 +3282,11 @@
       <c r="C55" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="56" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F55" s="24" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>107</v>
       </c>
@@ -3097,23 +3296,29 @@
       <c r="C56" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="57" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="F56" s="24" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>108</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F57" s="24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>38</v>
       </c>
-      <c r="H68" t="s">
+      <c r="I68" t="s">
         <v>39</v>
       </c>
-      <c r="M68" t="s">
+      <c r="N68" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>